<commit_message>
feat: Phase 9 adequacy batch, jobs API, and CRM UI updates
Add batch adequacy domain logic, scheduler job, Alembic migration, and tests.
Register dashboard and jobs routes; extend config, models, enums, and CRM schemas.

Remove client lines-of-business from the web UI (detail portfolio and import
guide), drop the LOB column from the import Excel template, and refresh PT
copy. Update Clients and Dashboard pages, docker-compose, and docs.

Co-Authored-By: Claude <noreply@anthropic.com>
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/importacao-clientes-modelo.xlsx
+++ b/apps/web/public/templates/importacao-clientes-modelo.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -447,10 +447,9 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="48" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,20 +510,15 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Linhas de negócio</t>
+          <t>Produtos detidos</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Produtos detidos</t>
+          <t>Perfil JSON</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Perfil JSON</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Segurados JSON</t>
         </is>
@@ -577,7 +571,6 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -590,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -755,64 +748,52 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Linhas de negócio</t>
+          <t>Produtos detidos</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Códigos na app, separados por vírgula ou ;. Vazio se não usar. Também: lob_codes.</t>
+          <t>Carteira: vários produtos separados por ;. Cada um: produto|seguradora|estado|início|fim (AAAA-MM-DD). Também: held_products.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Produtos detidos</t>
+          <t>Perfil JSON</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Carteira: vários produtos separados por ;. Cada um: produto|seguradora|estado|início|fim (AAAA-MM-DD). Também: held_products.</t>
+          <t>Avançado: JSON do perfil de seguros. Também: profile_json, perfil_json.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Perfil JSON</t>
+          <t>Segurados JSON</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Avançado: JSON do perfil de seguros. Também: profile_json, perfil_json.</t>
+          <t>Avançado: JSON com lista de segurados. Também: insured_persons_json, segurados_json.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Segurados JSON</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Avançado: JSON com lista de segurados. Também: insured_persons_json, segurados_json.</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-      <c r="B19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Validação</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Use Visualizar na aplicação antes de confirmar. Códigos LOB e nomes de produtos são validados com o catálogo da sua corretora.</t>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Use Visualizar na aplicação antes de confirmar. Nomes de produtos são validados com o catálogo da sua corretora.</t>
         </is>
       </c>
     </row>

</xml_diff>